<commit_message>
3-d variables and converting to local package
generating script for 3-d variables and converting repo structure to a local package for tranferability of additional species
</commit_message>
<xml_diff>
--- a/PacificHake/Table_A1_Pacific_Hake_Hypotheses.xlsx
+++ b/PacificHake/Table_A1_Pacific_Hake_Hypotheses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/megan.feddern/Documents/GitHub/mom6-based-groundfish-indices/PacificHake/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F68A06A-F2CC-C246-A2A6-2652AA4CEB64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F636BFD-7B6C-D842-B1F0-960337400521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table A1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1859" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1861" uniqueCount="400">
   <si>
     <t>TABLE A1: Pacific Hake (Merluccius productus) Conceptual Life History Model</t>
   </si>
@@ -1414,19 +1414,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1444,6 +1438,12 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -1451,17 +1451,7 @@
     <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1795,18 +1785,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
     </row>
     <row r="3" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -3532,34 +3522,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="4" customFormat="1" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -6396,37 +6386,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="7" t="s">
         <v>365</v>
       </c>
     </row>
@@ -7617,6 +7607,9 @@
       <c r="J37" t="s">
         <v>20</v>
       </c>
+      <c r="K37" t="s">
+        <v>373</v>
+      </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
@@ -7648,6 +7641,9 @@
       </c>
       <c r="J38" t="s">
         <v>20</v>
+      </c>
+      <c r="K38" t="s">
+        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -7655,7 +7651,7 @@
     <sortCondition ref="D1:D38"/>
   </sortState>
   <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Done">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Done">
       <formula>NOT(ISERROR(SEARCH("Done",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7674,153 +7670,153 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>376</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="8" t="s">
         <v>377</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="7" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>378</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="9" t="s">
         <v>379</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="9" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="12" t="s">
         <v>361</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="9" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="40" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>350</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>383</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="40" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="10" t="s">
         <v>357</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="9" t="s">
         <v>385</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="9" t="s">
         <v>387</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="9" t="s">
         <v>388</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="9" t="s">
         <v>389</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="9" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="40" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="9" t="s">
         <v>391</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="9" t="s">
         <v>392</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="9" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="100" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="9" t="s">
         <v>393</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="9" t="s">
         <v>394</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="9" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="9" t="s">
         <v>395</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="9" t="s">
         <v>396</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="9" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="80" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="9" t="s">
         <v>397</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="9" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="40" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="9" t="s">
         <v>398</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="9" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
     </row>
     <row r="25" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D25" t="s">

</xml_diff>